<commit_message>
feat(generator): drafts for REQ-008, REQ-009, REQ-010; questions and traceability
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/traceability.xlsx
+++ b/review/traceability.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="114">
   <si>
     <t>ID</t>
   </si>
@@ -194,6 +194,165 @@
   </si>
   <si>
     <t>Expenses CRUD in the database &gt; successful writes &gt; POST stores the regular user as owner when they create an expense</t>
+  </si>
+  <si>
+    <t>REQ-008</t>
+  </si>
+  <si>
+    <t>1 A regular user sees their own new expense in the list (control)</t>
+  </si>
+  <si>
+    <t>review/features/REQ-008.feature</t>
+  </si>
+  <si>
+    <t>review/specs/REQ-008.spec.ts</t>
+  </si>
+  <si>
+    <t>REQ-008 a regular user sees their own new expense in the list</t>
+  </si>
+  <si>
+    <t>2 A regular user's UI Export contains only their own expenses</t>
+  </si>
+  <si>
+    <t>REQ-008 a regular user's Export contains only their own expenses</t>
+  </si>
+  <si>
+    <t>BUG-001</t>
+  </si>
+  <si>
+    <t>fails (known defect)</t>
+  </si>
+  <si>
+    <t>3 A regular user's list filtered by category leaves out another user's expense</t>
+  </si>
+  <si>
+    <t>REQ-008 a regular user's list filtered by category leaves out another user's expense</t>
+  </si>
+  <si>
+    <t>AC1 list (API) shows only my expenses</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; GET list does not include another user's expense</t>
+  </si>
+  <si>
+    <t>AC1 export (API) shows only my expenses</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; export does not include another user's expense</t>
+  </si>
+  <si>
+    <t>AC1 detail (API) of another user's expense returns 403/404</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; GET returns 403 or 404 for another user's expense</t>
+  </si>
+  <si>
+    <t>AC1 detail (API) of my own expense returns 200 (control)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; a user can GET their own expense (control)</t>
+  </si>
+  <si>
+    <t>AC1 list (UI) as a regular user hides admin's expenses</t>
+  </si>
+  <si>
+    <t>tests/ui/expense-list.spec.ts</t>
+  </si>
+  <si>
+    <t>expense list &gt; as a regular user &gt; does not show admin's expenses @ui @regression</t>
+  </si>
+  <si>
+    <t>AC2 cannot edit another user's expense (API)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; PUT returns 403 or 404 for another user's expense and leaves it unchanged</t>
+  </si>
+  <si>
+    <t>AC2 cannot edit another user's expense (DB row unchanged)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD in the database &gt; rejected requests &gt; PUT by another user leaves the row unchanged</t>
+  </si>
+  <si>
+    <t>AC2 cannot delete another user's expense (API)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; another user's expense &gt; DELETE returns 403 or 404 for another user's expense and keeps it</t>
+  </si>
+  <si>
+    <t>AC2 cannot delete another user's expense (DB row kept)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD in the database &gt; rejected requests &gt; DELETE by another user keeps the row</t>
+  </si>
+  <si>
+    <t>REQ-009</t>
+  </si>
+  <si>
+    <t>1 Typing a unique title shows only matching rows</t>
+  </si>
+  <si>
+    <t>review/features/REQ-009.feature</t>
+  </si>
+  <si>
+    <t>review/specs/REQ-009.spec.ts</t>
+  </si>
+  <si>
+    <t>REQ-009 typing an expense's unique title shows only matching rows</t>
+  </si>
+  <si>
+    <t>fixme (planned)</t>
+  </si>
+  <si>
+    <t>2 Search ignores case</t>
+  </si>
+  <si>
+    <t>REQ-009 search ignores case</t>
+  </si>
+  <si>
+    <t>3 No match shows "No expenses found"</t>
+  </si>
+  <si>
+    <t>REQ-009 a search with no match shows "No expenses found"</t>
+  </si>
+  <si>
+    <t>REQ-010</t>
+  </si>
+  <si>
+    <t>1 Monthly total equals the sum of this month's rows shown</t>
+  </si>
+  <si>
+    <t>review/features/REQ-010.feature</t>
+  </si>
+  <si>
+    <t>review/specs/REQ-010.spec.ts</t>
+  </si>
+  <si>
+    <t>REQ-010 the monthly total equals the sum of this month's rows shown</t>
+  </si>
+  <si>
+    <t>2 An expense from another month is left out of the total</t>
+  </si>
+  <si>
+    <t>REQ-010 an expense from another month is left out of the total</t>
+  </si>
+  <si>
+    <t>3 Total includes an expense added this month</t>
+  </si>
+  <si>
+    <t>REQ-010 the total includes an expense added this month</t>
+  </si>
+  <si>
+    <t>4 Total follows an edited amount</t>
+  </si>
+  <si>
+    <t>REQ-010 the total follows an edited amount</t>
+  </si>
+  <si>
+    <t>5 Total drops a deleted expense</t>
+  </si>
+  <si>
+    <t>REQ-010 the total drops a deleted expense</t>
   </si>
 </sst>
 </file>
@@ -574,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1115,9 +1274,469 @@
         <v>12</v>
       </c>
     </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" t="s">
+        <v>68</v>
+      </c>
+      <c r="G25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C26" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" t="s">
+        <v>71</v>
+      </c>
+      <c r="F26" t="s">
+        <v>68</v>
+      </c>
+      <c r="G26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" t="s">
+        <v>73</v>
+      </c>
+      <c r="F27" t="s">
+        <v>68</v>
+      </c>
+      <c r="G27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+      <c r="F28" t="s">
+        <v>68</v>
+      </c>
+      <c r="G28" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" t="s">
+        <v>77</v>
+      </c>
+      <c r="F29" t="s">
+        <v>68</v>
+      </c>
+      <c r="G29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+      <c r="G30" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
+        <v>80</v>
+      </c>
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" t="s">
+        <v>82</v>
+      </c>
+      <c r="F31" t="s">
+        <v>68</v>
+      </c>
+      <c r="G31" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" t="s">
+        <v>84</v>
+      </c>
+      <c r="F32" t="s">
+        <v>68</v>
+      </c>
+      <c r="G32" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" t="s">
+        <v>59</v>
+      </c>
+      <c r="E33" t="s">
+        <v>86</v>
+      </c>
+      <c r="F33" t="s">
+        <v>68</v>
+      </c>
+      <c r="G33" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" t="s">
+        <v>88</v>
+      </c>
+      <c r="F34" t="s">
+        <v>68</v>
+      </c>
+      <c r="G34" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" t="s">
+        <v>89</v>
+      </c>
+      <c r="C35" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" t="s">
+        <v>68</v>
+      </c>
+      <c r="G35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>91</v>
+      </c>
+      <c r="B36" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+      <c r="G36" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>91</v>
+      </c>
+      <c r="B37" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" t="s">
+        <v>94</v>
+      </c>
+      <c r="E37" t="s">
+        <v>98</v>
+      </c>
+      <c r="F37" t="s">
+        <v>9</v>
+      </c>
+      <c r="G37" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" t="s">
+        <v>93</v>
+      </c>
+      <c r="D38" t="s">
+        <v>94</v>
+      </c>
+      <c r="E38" t="s">
+        <v>100</v>
+      </c>
+      <c r="F38" t="s">
+        <v>9</v>
+      </c>
+      <c r="G38" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" t="s">
+        <v>104</v>
+      </c>
+      <c r="E39" t="s">
+        <v>105</v>
+      </c>
+      <c r="F39" t="s">
+        <v>9</v>
+      </c>
+      <c r="G39" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" t="s">
+        <v>107</v>
+      </c>
+      <c r="F40" t="s">
+        <v>9</v>
+      </c>
+      <c r="G40" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B41" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" t="s">
+        <v>104</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" t="s">
+        <v>9</v>
+      </c>
+      <c r="G41" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>101</v>
+      </c>
+      <c r="B42" t="s">
+        <v>110</v>
+      </c>
+      <c r="C42" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" t="s">
+        <v>104</v>
+      </c>
+      <c r="E42" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" t="s">
+        <v>9</v>
+      </c>
+      <c r="G42" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B43" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" t="s">
+        <v>104</v>
+      </c>
+      <c r="E43" t="s">
+        <v>113</v>
+      </c>
+      <c r="F43" t="s">
+        <v>9</v>
+      </c>
+      <c r="G43" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test: promote REQ-002 drafts into the suite
- api: boundary loop now validates the body schema and covers 999999.99, future
  and old dates and all six categories (draft scenarios 16-18, 27, 29-30); missing
  fields, -0.01, "1,000" and "12,50" join the validation table
- db: the same values in the stored/rejected loops; duplicate POST stores two rows
- ui: required-field, boundary-amount, future-date, duplicate and dropdown tests in
  expense-crud; new "success message" block; date and same-date order in expense-list
- review/specs/REQ-002.spec.ts removed; traceability rows point to the suite tests
  with status "approved, in suite"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/traceability.xlsx
+++ b/review/traceability.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="185">
   <si>
     <t>ID</t>
   </si>
@@ -58,369 +58,375 @@
     <t>review/features/REQ-002.feature</t>
   </si>
   <si>
-    <t>review/specs/REQ-002.spec.ts</t>
-  </si>
-  <si>
-    <t>REQ-002 leaving only title empty shows "Title is required" and stores nothing</t>
+    <t>expense CRUD &gt; form validation &gt; leaving only title empty shows "Title is required" and stores nothing @ui @regression</t>
+  </si>
+  <si>
+    <t>approved, in suite</t>
+  </si>
+  <si>
+    <t>3 Only amount empty shows its required message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; leaving only amount empty shows "Amount is required" and stores nothing @ui @regression</t>
+  </si>
+  <si>
+    <t>4 Only category empty shows its required message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; leaving only category empty shows "Category is required" and stores nothing @ui @regression</t>
+  </si>
+  <si>
+    <t>5 Only date empty shows its required message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; leaving only date empty shows "Date is required" and stores nothing @ui @regression</t>
+  </si>
+  <si>
+    <t>6 POST without title returns 400</t>
+  </si>
+  <si>
+    <t>tests/api/expenses.spec.ts</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when title is missing</t>
+  </si>
+  <si>
+    <t>7 POST without amount returns 400</t>
+  </si>
+  <si>
+    <t>tests/api/expenses.spec.ts + tests/db/expenses.spec.ts</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is missing + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when amount is missing</t>
+  </si>
+  <si>
+    <t>8 POST without category returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when category is missing + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when category is missing</t>
+  </si>
+  <si>
+    <t>9 POST without date returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date is missing + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when date is missing</t>
+  </si>
+  <si>
+    <t>10 POST with a numeric title returns "Title must be a string"</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 "Title must be a string" when title is a number</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>12 POST with amount 0 returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is zero</t>
+  </si>
+  <si>
+    <t>13 POST with amount -0.01 returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is -0.01 + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when amount is -0.01</t>
+  </si>
+  <si>
+    <t>14 POST with amount 1000000.01 returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is above 1000000</t>
+  </si>
+  <si>
+    <t>15 POST with amount 1.234 returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount has 3 decimal places</t>
+  </si>
+  <si>
+    <t>16 POST with amount 0.01 returns 201, stored exactly</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for the minimum amount 0.01 + Expenses CRUD in the database &gt; successful writes &gt; POST stores the minimum amount 0.01 exactly</t>
+  </si>
+  <si>
+    <t>17 POST with amount 1000000 returns 201, stored exactly</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for the maximum amount 1000000 + Expenses CRUD in the database &gt; successful writes &gt; POST stores the maximum amount 1000000 exactly</t>
+  </si>
+  <si>
+    <t>18 POST with amount 999999.99 returns 201, stored exactly</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for the amount 999999.99 + Expenses CRUD in the database &gt; successful writes &gt; POST stores the amount 999999.99 exactly</t>
+  </si>
+  <si>
+    <t>19 UI add with amount 0.01 shows $0.01</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; adding amount 0.01 shows "Expense added" and a row with $0.01 @ui @regression</t>
+  </si>
+  <si>
+    <t>20 UI add with amount 1000000 shows $1,000,000.00</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; adding amount 1000000 shows "Expense added" and a row with $1,000,000.00 @ui @regression</t>
+  </si>
+  <si>
+    <t>22 Adding a valid expense shows "Expense added" and the new row (DB checked)</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; adding an expense shows "Expense added" and the new row @smoke @ui</t>
+  </si>
+  <si>
+    <t>23 New row appears once without reload; count matches the list; one row stored in the DB</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; the new row appears once without a page reload and the count matches the list @ui @regression</t>
+  </si>
+  <si>
+    <t>24 A regular user's expense is stored with them as owner</t>
+  </si>
+  <si>
+    <t>tests/db/expenses.spec.ts</t>
+  </si>
+  <si>
+    <t>Expenses CRUD in the database &gt; successful writes &gt; POST stores the regular user as owner when they create an expense</t>
+  </si>
+  <si>
+    <t>C2 POST with a whitespace-only title returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when title is only whitespace</t>
+  </si>
+  <si>
+    <t>C2 POST with a 201-character title returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when title is longer than 200 characters</t>
+  </si>
+  <si>
+    <t>C2 POST with a 200-character title returns 201</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for a 200-character title</t>
+  </si>
+  <si>
+    <t>C2 UI whitespace-only title shows "Title is required"</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; a whitespace-only title shows "Title is required" @ui @regression</t>
+  </si>
+  <si>
+    <t>C2 UI 201-character title is rejected</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; a 201-character title shows "Title must be at most 200 characters" and stores nothing @ui @regression</t>
+  </si>
+  <si>
+    <t>C4 POST accepts a dot-decimal amount string (12.50)</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST trims the title and accepts a numeric-string amount</t>
+  </si>
+  <si>
+    <t>25 POST with amount "1,000" returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount has a thousands separator ("1,000") + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when amount has a thousands separator ("1,000")</t>
+  </si>
+  <si>
+    <t>26 POST with amount "12,50" returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount has a decimal comma ("12,50") + Expenses CRUD in the database &gt; rejected requests &gt; POST inserts no row when amount has a decimal comma ("12,50")</t>
+  </si>
+  <si>
+    <t>27 POST with category Food returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Food + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Food exactly</t>
+  </si>
+  <si>
+    <t>27 POST with category Travel returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Travel + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Travel exactly</t>
+  </si>
+  <si>
+    <t>27 POST with category Office returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Office + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Office exactly</t>
+  </si>
+  <si>
+    <t>27 POST with category Utilities returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Utilities + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Utilities exactly</t>
+  </si>
+  <si>
+    <t>27 POST with category Entertainment returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Entertainment + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Entertainment exactly</t>
+  </si>
+  <si>
+    <t>27 POST with category Other returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for category Other + Expenses CRUD in the database &gt; successful writes &gt; POST stores category Other exactly</t>
+  </si>
+  <si>
+    <t>C5 POST with an unknown category returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when category is not allowed</t>
+  </si>
+  <si>
+    <t>C5 POST with a wrong-case category returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when category has the wrong case</t>
+  </si>
+  <si>
+    <t>28 Category dropdown offers exactly the six categories</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; form validation &gt; the category dropdown offers exactly the six categories @ui @regression</t>
+  </si>
+  <si>
+    <t>29 POST with a future date returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for a future date + Expenses CRUD in the database &gt; successful writes &gt; POST stores a future date exactly</t>
+  </si>
+  <si>
+    <t>30 POST with an old date returns 201, stored</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for an old date + Expenses CRUD in the database &gt; successful writes &gt; POST stores an old date exactly</t>
+  </si>
+  <si>
+    <t>31 UI add with a future date shows the row</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; adding an expense with a future date shows it in the list @ui @regression</t>
+  </si>
+  <si>
+    <t>C6 POST with a nonexistent date returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date does not exist</t>
+  </si>
+  <si>
+    <t>C6 POST with a DD/MM/YYYY date returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date is DD/MM/YYYY</t>
+  </si>
+  <si>
+    <t>C6 POST with a non-zero-padded date returns 400</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date is not zero-padded</t>
+  </si>
+  <si>
+    <t>C6 POST with a leap-day date returns 201</t>
+  </si>
+  <si>
+    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for a leap-day date</t>
+  </si>
+  <si>
+    <t>32 POST the same expense twice stores two rows</t>
+  </si>
+  <si>
+    <t>Expenses CRUD in the database &gt; successful writes &gt; POSTing the same expense twice stores two rows</t>
+  </si>
+  <si>
+    <t>33 UI add the same expense twice shows two rows</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; add &gt; adding the same expense twice shows two rows @ui @regression</t>
+  </si>
+  <si>
+    <t>34 "Expense added" still shown 10 minutes later</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; "Expense added" is still shown 10 minutes later with no action @ui @regression</t>
+  </si>
+  <si>
+    <t>35 Opening the Add form hides the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; opening the Add form hides the success message @ui @regression</t>
+  </si>
+  <si>
+    <t>36 A back-dated new expense appears in date order</t>
+  </si>
+  <si>
+    <t>tests/ui/expense-list.spec.ts</t>
+  </si>
+  <si>
+    <t>expense list &gt; with data &gt; a back-dated new expense appears in date order @ui @regression</t>
+  </si>
+  <si>
+    <t>37 Opening Edit hides the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; opening Edit hides the success message @ui @regression</t>
+  </si>
+  <si>
+    <t>38 An error message replaces the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; an error message replaces the success message @ui @regression</t>
+  </si>
+  <si>
+    <t>39 Filtering by category keeps the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; filtering by category keeps the success message @ui @regression</t>
+  </si>
+  <si>
+    <t>40 Export keeps the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; Export keeps the success message @ui @file @regression</t>
+  </si>
+  <si>
+    <t>41 Import keeps the success message</t>
+  </si>
+  <si>
+    <t>expense CRUD &gt; success message &gt; Import keeps the success message @ui @file @regression</t>
+  </si>
+  <si>
+    <t>42 Same date: the newer expense is listed first</t>
+  </si>
+  <si>
+    <t>expense list &gt; with data &gt; on the same date the newer expense is listed first @ui @regression</t>
+  </si>
+  <si>
+    <t>REQ-008</t>
+  </si>
+  <si>
+    <t>1 A regular user sees their own new expense in the list (control)</t>
+  </si>
+  <si>
+    <t>review/features/REQ-008.feature</t>
+  </si>
+  <si>
+    <t>review/specs/REQ-008.spec.ts</t>
+  </si>
+  <si>
+    <t>REQ-008 a regular user sees their own new expense in the list</t>
   </si>
   <si>
     <t>passes</t>
   </si>
   <si>
-    <t>3 Only amount empty shows its required message</t>
-  </si>
-  <si>
-    <t>REQ-002 leaving only amount empty shows "Amount is required" and stores nothing</t>
-  </si>
-  <si>
-    <t>4 Only category empty shows its required message</t>
-  </si>
-  <si>
-    <t>REQ-002 leaving only category empty shows "Category is required" and stores nothing</t>
-  </si>
-  <si>
-    <t>5 Only date empty shows its required message</t>
-  </si>
-  <si>
-    <t>REQ-002 leaving only date empty shows "Date is required" and stores nothing</t>
-  </si>
-  <si>
-    <t>6 POST without title returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST without title returns 400 naming only title</t>
-  </si>
-  <si>
-    <t>7 POST without amount returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST without amount returns 400 naming only amount</t>
-  </si>
-  <si>
-    <t>8 POST without category returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST without category returns 400 naming only category</t>
-  </si>
-  <si>
-    <t>9 POST without date returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST without date returns 400 naming only date</t>
-  </si>
-  <si>
-    <t>10 POST with a numeric title returns "Title must be a string"</t>
-  </si>
-  <si>
-    <t>tests/api/expenses.spec.ts</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 "Title must be a string" when title is a number</t>
-  </si>
-  <si>
-    <t>BUG-002</t>
-  </si>
-  <si>
-    <t>12 POST with amount 0 returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is zero</t>
-  </si>
-  <si>
-    <t>13 POST with amount -0.01 returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount -0.01 returns 400 "Amount must be greater than 0"</t>
-  </si>
-  <si>
-    <t>14 POST with amount 1000000.01 returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount is above 1000000</t>
-  </si>
-  <si>
-    <t>15 POST with amount 1.234 returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when amount has 3 decimal places</t>
-  </si>
-  <si>
-    <t>16 POST with amount 0.01 returns 201, stored exactly</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount 0.01 returns 201 and stores it exactly</t>
-  </si>
-  <si>
-    <t>17 POST with amount 1000000 returns 201, stored exactly</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount 1000000 returns 201 and stores it exactly</t>
-  </si>
-  <si>
-    <t>18 POST with amount 999999.99 returns 201, stored exactly</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount 999999.99 returns 201 and stores it exactly</t>
-  </si>
-  <si>
-    <t>19 UI add with amount 0.01 shows $0.01</t>
-  </si>
-  <si>
-    <t>REQ-002 adding amount 0.01 shows "Expense added" and a row with $0.01</t>
-  </si>
-  <si>
-    <t>20 UI add with amount 1000000 shows $1,000,000.00</t>
-  </si>
-  <si>
-    <t>REQ-002 adding amount 1000000 shows "Expense added" and a row with $1,000,000.00</t>
-  </si>
-  <si>
-    <t>22 Adding a valid expense shows "Expense added" and the new row (DB checked)</t>
-  </si>
-  <si>
-    <t>expense CRUD &gt; add &gt; adding an expense shows "Expense added" and the new row @smoke @ui</t>
-  </si>
-  <si>
-    <t>23 New row appears once without reload; count matches the list; one row stored in the DB</t>
-  </si>
-  <si>
-    <t>REQ-002 the new row appears once without a page reload and the count matches the list</t>
-  </si>
-  <si>
-    <t>24 A regular user's expense is stored with them as owner</t>
-  </si>
-  <si>
-    <t>tests/db/expenses.spec.ts</t>
-  </si>
-  <si>
-    <t>Expenses CRUD in the database &gt; successful writes &gt; POST stores the regular user as owner when they create an expense</t>
-  </si>
-  <si>
-    <t>C2 POST with a whitespace-only title returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when title is only whitespace</t>
-  </si>
-  <si>
-    <t>C2 POST with a 201-character title returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when title is longer than 200 characters</t>
-  </si>
-  <si>
-    <t>C2 POST with a 200-character title returns 201</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for a 200-character title</t>
-  </si>
-  <si>
-    <t>C2 UI whitespace-only title shows "Title is required"</t>
-  </si>
-  <si>
-    <t>expense CRUD &gt; form validation &gt; a whitespace-only title shows "Title is required" @ui @regression</t>
-  </si>
-  <si>
-    <t>C2 UI 201-character title is rejected</t>
-  </si>
-  <si>
-    <t>expense CRUD &gt; form validation &gt; a 201-character title shows "Title must be at most 200 characters" and stores nothing @ui @regression</t>
-  </si>
-  <si>
-    <t>C4 POST accepts a dot-decimal amount string (12.50)</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; happy path &gt; POST trims the title and accepts a numeric-string amount</t>
-  </si>
-  <si>
-    <t>25 POST with amount "1,000" returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount "1,000" returns 400 "Amount must be a number" and stores nothing</t>
-  </si>
-  <si>
-    <t>26 POST with amount "12,50" returns 400</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with amount "12,50" returns 400 "Amount must be a number" and stores nothing</t>
-  </si>
-  <si>
-    <t>27 POST with category Food returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Food returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>27 POST with category Travel returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Travel returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>27 POST with category Office returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Office returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>27 POST with category Utilities returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Utilities returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>27 POST with category Entertainment returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Entertainment returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>27 POST with category Other returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with category Other returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>C5 POST with an unknown category returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when category is not allowed</t>
-  </si>
-  <si>
-    <t>C5 POST with a wrong-case category returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when category has the wrong case</t>
-  </si>
-  <si>
-    <t>28 Category dropdown offers exactly the six categories</t>
-  </si>
-  <si>
-    <t>REQ-002 the category dropdown offers exactly the six categories</t>
-  </si>
-  <si>
-    <t>29 POST with a future date returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with a future date (2099-12-31) returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>30 POST with an old date returns 201, stored</t>
-  </si>
-  <si>
-    <t>REQ-002 POST with an old date (1900-01-01) returns 201 and stores it</t>
-  </si>
-  <si>
-    <t>31 UI add with a future date shows the row</t>
-  </si>
-  <si>
-    <t>REQ-002 adding an expense with a future date shows it in the list</t>
-  </si>
-  <si>
-    <t>C6 POST with a nonexistent date returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date does not exist</t>
-  </si>
-  <si>
-    <t>C6 POST with a DD/MM/YYYY date returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date is DD/MM/YYYY</t>
-  </si>
-  <si>
-    <t>C6 POST with a non-zero-padded date returns 400</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; validation &gt; POST returns 400 when date is not zero-padded</t>
-  </si>
-  <si>
-    <t>C6 POST with a leap-day date returns 201</t>
-  </si>
-  <si>
-    <t>Expenses CRUD &gt; happy path &gt; POST returns 201 for a leap-day date</t>
-  </si>
-  <si>
-    <t>32 POST the same expense twice stores two rows</t>
-  </si>
-  <si>
-    <t>REQ-002 POSTing the same expense twice returns 201 twice and stores two rows</t>
-  </si>
-  <si>
-    <t>33 UI add the same expense twice shows two rows</t>
-  </si>
-  <si>
-    <t>REQ-002 adding the same expense twice shows two rows</t>
-  </si>
-  <si>
-    <t>34 "Expense added" still shown 10 minutes later</t>
-  </si>
-  <si>
-    <t>REQ-002 "Expense added" is still shown 10 minutes later with no action</t>
-  </si>
-  <si>
-    <t>35 Opening the Add form hides the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 opening the Add form hides the success message</t>
-  </si>
-  <si>
-    <t>36 A back-dated new expense appears in date order</t>
-  </si>
-  <si>
-    <t>REQ-002 a back-dated new expense appears in date order</t>
-  </si>
-  <si>
-    <t>37 Opening Edit hides the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 opening Edit hides the success message</t>
-  </si>
-  <si>
-    <t>38 An error message replaces the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 an error message replaces the success message</t>
-  </si>
-  <si>
-    <t>39 Filtering by category keeps the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 filtering by category keeps the success message</t>
-  </si>
-  <si>
-    <t>40 Export keeps the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 Export keeps the success message</t>
-  </si>
-  <si>
-    <t>41 Import keeps the success message</t>
-  </si>
-  <si>
-    <t>REQ-002 Import keeps the success message</t>
-  </si>
-  <si>
-    <t>42 Same date: the newer expense is listed first</t>
-  </si>
-  <si>
-    <t>REQ-002 on the same date the newer expense is listed first</t>
-  </si>
-  <si>
-    <t>REQ-008</t>
-  </si>
-  <si>
-    <t>1 A regular user sees their own new expense in the list (control)</t>
-  </si>
-  <si>
-    <t>review/features/REQ-008.feature</t>
-  </si>
-  <si>
-    <t>review/specs/REQ-008.spec.ts</t>
-  </si>
-  <si>
-    <t>REQ-008 a regular user sees their own new expense in the list</t>
-  </si>
-  <si>
     <t>2 A regular user's UI Export contains only their own expenses</t>
   </si>
   <si>
@@ -464,9 +470,6 @@
   </si>
   <si>
     <t>AC1 list (UI) as a regular user hides admin's expenses</t>
-  </si>
-  <si>
-    <t>tests/ui/expense-list.spec.ts</t>
   </si>
   <si>
     <t>expense list &gt; as a regular user &gt; does not show admin's expenses @ui @regression</t>
@@ -1012,16 +1015,16 @@
         <v>14</v>
       </c>
       <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
       <c r="F3" t="s">
         <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1029,22 +1032,22 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
       <c r="F4" t="s">
         <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1052,22 +1055,22 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
       <c r="F5" t="s">
         <v>9</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1075,22 +1078,22 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
       <c r="F6" t="s">
         <v>9</v>
       </c>
       <c r="G6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1098,13 +1101,13 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
         <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>15</v>
       </c>
       <c r="E7" t="s">
         <v>25</v>
@@ -1113,7 +1116,7 @@
         <v>9</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1127,16 +1130,16 @@
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1144,22 +1147,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1167,22 +1170,22 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1190,13 +1193,13 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
         <v>34</v>
@@ -1219,7 +1222,7 @@
         <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
         <v>37</v>
@@ -1242,7 +1245,7 @@
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
         <v>39</v>
@@ -1251,7 +1254,7 @@
         <v>9</v>
       </c>
       <c r="G13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1265,7 +1268,7 @@
         <v>9</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
         <v>41</v>
@@ -1288,7 +1291,7 @@
         <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E15" t="s">
         <v>43</v>
@@ -1311,7 +1314,7 @@
         <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E16" t="s">
         <v>45</v>
@@ -1320,7 +1323,7 @@
         <v>9</v>
       </c>
       <c r="G16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1334,7 +1337,7 @@
         <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E17" t="s">
         <v>47</v>
@@ -1343,7 +1346,7 @@
         <v>9</v>
       </c>
       <c r="G17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1357,7 +1360,7 @@
         <v>14</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E18" t="s">
         <v>49</v>
@@ -1366,7 +1369,7 @@
         <v>9</v>
       </c>
       <c r="G18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1380,7 +1383,7 @@
         <v>14</v>
       </c>
       <c r="D19" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E19" t="s">
         <v>51</v>
@@ -1389,7 +1392,7 @@
         <v>9</v>
       </c>
       <c r="G19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1403,7 +1406,7 @@
         <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
@@ -1412,7 +1415,7 @@
         <v>9</v>
       </c>
       <c r="G20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1449,7 +1452,7 @@
         <v>14</v>
       </c>
       <c r="D22" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s">
         <v>57</v>
@@ -1458,7 +1461,7 @@
         <v>9</v>
       </c>
       <c r="G22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1495,7 +1498,7 @@
         <v>9</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E24" t="s">
         <v>62</v>
@@ -1518,7 +1521,7 @@
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E25" t="s">
         <v>64</v>
@@ -1541,7 +1544,7 @@
         <v>9</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E26" t="s">
         <v>66</v>
@@ -1610,7 +1613,7 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E29" t="s">
         <v>72</v>
@@ -1633,7 +1636,7 @@
         <v>14</v>
       </c>
       <c r="D30" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E30" t="s">
         <v>74</v>
@@ -1642,7 +1645,7 @@
         <v>9</v>
       </c>
       <c r="G30" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1656,7 +1659,7 @@
         <v>14</v>
       </c>
       <c r="D31" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E31" t="s">
         <v>76</v>
@@ -1665,7 +1668,7 @@
         <v>9</v>
       </c>
       <c r="G31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1679,7 +1682,7 @@
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E32" t="s">
         <v>78</v>
@@ -1688,7 +1691,7 @@
         <v>9</v>
       </c>
       <c r="G32" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -1702,7 +1705,7 @@
         <v>14</v>
       </c>
       <c r="D33" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E33" t="s">
         <v>80</v>
@@ -1711,7 +1714,7 @@
         <v>9</v>
       </c>
       <c r="G33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -1725,7 +1728,7 @@
         <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E34" t="s">
         <v>82</v>
@@ -1734,7 +1737,7 @@
         <v>9</v>
       </c>
       <c r="G34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -1748,7 +1751,7 @@
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E35" t="s">
         <v>84</v>
@@ -1757,7 +1760,7 @@
         <v>9</v>
       </c>
       <c r="G35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -1771,7 +1774,7 @@
         <v>14</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E36" t="s">
         <v>86</v>
@@ -1780,7 +1783,7 @@
         <v>9</v>
       </c>
       <c r="G36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -1794,7 +1797,7 @@
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E37" t="s">
         <v>88</v>
@@ -1803,7 +1806,7 @@
         <v>9</v>
       </c>
       <c r="G37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -1817,7 +1820,7 @@
         <v>9</v>
       </c>
       <c r="D38" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E38" t="s">
         <v>90</v>
@@ -1840,7 +1843,7 @@
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E39" t="s">
         <v>92</v>
@@ -1863,7 +1866,7 @@
         <v>14</v>
       </c>
       <c r="D40" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E40" t="s">
         <v>94</v>
@@ -1872,7 +1875,7 @@
         <v>9</v>
       </c>
       <c r="G40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -1886,7 +1889,7 @@
         <v>14</v>
       </c>
       <c r="D41" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E41" t="s">
         <v>96</v>
@@ -1895,7 +1898,7 @@
         <v>9</v>
       </c>
       <c r="G41" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -1909,7 +1912,7 @@
         <v>14</v>
       </c>
       <c r="D42" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E42" t="s">
         <v>98</v>
@@ -1918,7 +1921,7 @@
         <v>9</v>
       </c>
       <c r="G42" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1932,7 +1935,7 @@
         <v>14</v>
       </c>
       <c r="D43" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E43" t="s">
         <v>100</v>
@@ -1941,7 +1944,7 @@
         <v>9</v>
       </c>
       <c r="G43" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
@@ -1955,7 +1958,7 @@
         <v>9</v>
       </c>
       <c r="D44" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E44" t="s">
         <v>102</v>
@@ -1978,7 +1981,7 @@
         <v>9</v>
       </c>
       <c r="D45" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E45" t="s">
         <v>104</v>
@@ -2001,7 +2004,7 @@
         <v>9</v>
       </c>
       <c r="D46" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E46" t="s">
         <v>106</v>
@@ -2024,7 +2027,7 @@
         <v>9</v>
       </c>
       <c r="D47" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E47" t="s">
         <v>108</v>
@@ -2047,7 +2050,7 @@
         <v>14</v>
       </c>
       <c r="D48" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="E48" t="s">
         <v>110</v>
@@ -2056,7 +2059,7 @@
         <v>9</v>
       </c>
       <c r="G48" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
@@ -2070,7 +2073,7 @@
         <v>14</v>
       </c>
       <c r="D49" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E49" t="s">
         <v>112</v>
@@ -2079,7 +2082,7 @@
         <v>9</v>
       </c>
       <c r="G49" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
@@ -2093,7 +2096,7 @@
         <v>14</v>
       </c>
       <c r="D50" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E50" t="s">
         <v>114</v>
@@ -2102,7 +2105,7 @@
         <v>9</v>
       </c>
       <c r="G50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
@@ -2116,7 +2119,7 @@
         <v>14</v>
       </c>
       <c r="D51" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E51" t="s">
         <v>116</v>
@@ -2125,7 +2128,7 @@
         <v>9</v>
       </c>
       <c r="G51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
@@ -2139,16 +2142,16 @@
         <v>14</v>
       </c>
       <c r="D52" t="s">
-        <v>15</v>
+        <v>118</v>
       </c>
       <c r="E52" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F52" t="s">
         <v>9</v>
       </c>
       <c r="G52" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
@@ -2156,22 +2159,22 @@
         <v>7</v>
       </c>
       <c r="B53" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C53" t="s">
         <v>14</v>
       </c>
       <c r="D53" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E53" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F53" t="s">
         <v>9</v>
       </c>
       <c r="G53" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
@@ -2179,22 +2182,22 @@
         <v>7</v>
       </c>
       <c r="B54" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C54" t="s">
         <v>14</v>
       </c>
       <c r="D54" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E54" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F54" t="s">
         <v>9</v>
       </c>
       <c r="G54" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
@@ -2202,22 +2205,22 @@
         <v>7</v>
       </c>
       <c r="B55" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C55" t="s">
         <v>14</v>
       </c>
       <c r="D55" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E55" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F55" t="s">
         <v>9</v>
       </c>
       <c r="G55" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
@@ -2225,22 +2228,22 @@
         <v>7</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C56" t="s">
         <v>14</v>
       </c>
       <c r="D56" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F56" t="s">
         <v>9</v>
       </c>
       <c r="G56" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -2248,22 +2251,22 @@
         <v>7</v>
       </c>
       <c r="B57" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C57" t="s">
         <v>14</v>
       </c>
       <c r="D57" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E57" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F57" t="s">
         <v>9</v>
       </c>
       <c r="G57" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
@@ -2271,111 +2274,111 @@
         <v>7</v>
       </c>
       <c r="B58" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C58" t="s">
         <v>14</v>
       </c>
       <c r="D58" t="s">
-        <v>15</v>
+        <v>118</v>
       </c>
       <c r="E58" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F58" t="s">
         <v>9</v>
       </c>
       <c r="G58" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B59" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C59" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D59" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E59" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F59" t="s">
         <v>9</v>
       </c>
       <c r="G59" t="s">
-        <v>17</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B60" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C60" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D60" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E60" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F60" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G60" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B61" t="s">
+        <v>142</v>
+      </c>
+      <c r="C61" t="s">
+        <v>134</v>
+      </c>
+      <c r="D61" t="s">
+        <v>135</v>
+      </c>
+      <c r="E61" t="s">
+        <v>143</v>
+      </c>
+      <c r="F61" t="s">
         <v>140</v>
       </c>
-      <c r="C61" t="s">
-        <v>133</v>
-      </c>
-      <c r="D61" t="s">
-        <v>134</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="G61" t="s">
         <v>141</v>
-      </c>
-      <c r="F61" t="s">
-        <v>138</v>
-      </c>
-      <c r="G61" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B62" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C62" t="s">
         <v>9</v>
       </c>
       <c r="D62" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E62" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F62" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G62" t="s">
         <v>12</v>
@@ -2383,22 +2386,22 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B63" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C63" t="s">
         <v>9</v>
       </c>
       <c r="D63" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E63" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F63" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G63" t="s">
         <v>12</v>
@@ -2406,22 +2409,22 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B64" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C64" t="s">
         <v>9</v>
       </c>
       <c r="D64" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E64" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F64" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G64" t="s">
         <v>12</v>
@@ -2429,19 +2432,19 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B65" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C65" t="s">
         <v>9</v>
       </c>
       <c r="D65" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E65" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F65" t="s">
         <v>9</v>
@@ -2452,22 +2455,22 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B66" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C66" t="s">
         <v>9</v>
       </c>
       <c r="D66" t="s">
-        <v>151</v>
+        <v>118</v>
       </c>
       <c r="E66" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F66" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G66" t="s">
         <v>12</v>
@@ -2475,22 +2478,22 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B67" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C67" t="s">
         <v>9</v>
       </c>
       <c r="D67" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E67" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F67" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G67" t="s">
         <v>12</v>
@@ -2498,10 +2501,10 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B68" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C68" t="s">
         <v>9</v>
@@ -2510,10 +2513,10 @@
         <v>59</v>
       </c>
       <c r="E68" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F68" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G68" t="s">
         <v>12</v>
@@ -2521,22 +2524,22 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B69" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C69" t="s">
         <v>9</v>
       </c>
       <c r="D69" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E69" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F69" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G69" t="s">
         <v>12</v>
@@ -2544,10 +2547,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B70" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C70" t="s">
         <v>9</v>
@@ -2556,10 +2559,10 @@
         <v>59</v>
       </c>
       <c r="E70" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F70" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G70" t="s">
         <v>12</v>
@@ -2567,191 +2570,191 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B71" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C71" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D71" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F71" t="s">
         <v>9</v>
       </c>
       <c r="G71" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B72" t="s">
+        <v>168</v>
+      </c>
+      <c r="C72" t="s">
+        <v>164</v>
+      </c>
+      <c r="D72" t="s">
+        <v>165</v>
+      </c>
+      <c r="E72" t="s">
+        <v>169</v>
+      </c>
+      <c r="F72" t="s">
+        <v>9</v>
+      </c>
+      <c r="G72" t="s">
         <v>167</v>
-      </c>
-      <c r="C72" t="s">
-        <v>163</v>
-      </c>
-      <c r="D72" t="s">
-        <v>164</v>
-      </c>
-      <c r="E72" t="s">
-        <v>168</v>
-      </c>
-      <c r="F72" t="s">
-        <v>9</v>
-      </c>
-      <c r="G72" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B73" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C73" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D73" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E73" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F73" t="s">
         <v>9</v>
       </c>
       <c r="G73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B74" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C74" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D74" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F74" t="s">
         <v>9</v>
       </c>
       <c r="G74" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B75" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C75" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D75" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E75" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F75" t="s">
         <v>9</v>
       </c>
       <c r="G75" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B76" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D76" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E76" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F76" t="s">
         <v>9</v>
       </c>
       <c r="G76" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B77" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C77" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D77" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E77" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F77" t="s">
         <v>9</v>
       </c>
       <c r="G77" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B78" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C78" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D78" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E78" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F78" t="s">
         <v>9</v>
       </c>
       <c r="G78" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>